<commit_message>
Update Excel transaction files with new data and add a new file
- Updated existing Excel files for transactions to reflect recent changes.
- Added a new Excel file for transactions to enhance data tracking and reporting capabilities.
</commit_message>
<xml_diff>
--- a/data/transactions/أذونات الإضافة لشهر 3.xlsx
+++ b/data/transactions/أذونات الإضافة لشهر 3.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\ERP\Development\erp-server\data\transactions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7868058F-C819-45A2-ABE4-7FB72E40C1C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3313370A-44D2-4BE8-96D1-1216B10DD512}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="15600" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2504,7 +2504,7 @@
   <cols>
     <col min="1" max="1" width="6.5703125" customWidth="1"/>
     <col min="2" max="2" width="16.5703125" customWidth="1"/>
-    <col min="3" max="3" width="31.28515625" customWidth="1"/>
+    <col min="3" max="3" width="50.7109375" customWidth="1"/>
     <col min="4" max="4" width="8.140625" customWidth="1"/>
     <col min="5" max="5" width="11.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.85546875" customWidth="1"/>

</xml_diff>

<commit_message>
Update Excel transaction files with revised data for transactions 3 and 6
</commit_message>
<xml_diff>
--- a/data/transactions/أذونات الإضافة لشهر 3.xlsx
+++ b/data/transactions/أذونات الإضافة لشهر 3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\ERP\Development\erp-server\data\transactions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2919998B-695B-424F-98C5-82759DDC1C45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{613BD2F1-EC05-4427-AD69-6D4D1F68C8B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2013" uniqueCount="774">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2012" uniqueCount="775">
   <si>
     <t>بورسعيد لصناعة المعادن</t>
   </si>
@@ -2359,6 +2359,9 @@
   </si>
   <si>
     <t>متر 3</t>
+  </si>
+  <si>
+    <t>10307010</t>
   </si>
 </sst>
 </file>
@@ -4817,7 +4820,7 @@
         <v>45</v>
       </c>
       <c r="B51" s="12" t="s">
-        <v>158</v>
+        <v>774</v>
       </c>
       <c r="C51" s="7" t="s">
         <v>105</v>
@@ -13959,9 +13962,7 @@
       <c r="A286" s="1">
         <v>280</v>
       </c>
-      <c r="B286" s="9" t="s">
-        <v>540</v>
-      </c>
+      <c r="B286" s="9"/>
       <c r="C286" s="7" t="s">
         <v>516</v>
       </c>

</xml_diff>